<commit_message>
Leave signature columns blank in attendance sheet
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01LsGdck9uUBqMn7Bw6wMhA5
</commit_message>
<xml_diff>
--- a/Personel_Devam_Cizelgesi_Eylul_2026_SULEYMAN_YILDIZ.xlsx
+++ b/Personel_Devam_Cizelgesi_Eylul_2026_SULEYMAN_YILDIZ.xlsx
@@ -399,7 +399,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="42">
+  <cellXfs count="40">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="11" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -486,12 +486,6 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="14" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="12" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1487,11 +1481,7 @@
           <t>01:00</t>
         </is>
       </c>
-      <c r="D35" s="40" t="inlineStr">
-        <is>
-          <t>SULEYMAN YILDIZ</t>
-        </is>
-      </c>
+      <c r="D35" s="6" t="n"/>
       <c r="E35" s="6" t="n"/>
       <c r="F35" s="6" t="n"/>
       <c r="G35" s="6" t="n"/>
@@ -1501,11 +1491,7 @@
           <t>09:00</t>
         </is>
       </c>
-      <c r="J35" s="41" t="inlineStr">
-        <is>
-          <t>SULEYMAN YILDIZ</t>
-        </is>
-      </c>
+      <c r="J35" s="9" t="n"/>
       <c r="K35" s="10" t="n"/>
     </row>
     <row r="36" ht="21.75" customHeight="1">
@@ -1517,11 +1503,7 @@
           <t>01:00</t>
         </is>
       </c>
-      <c r="D36" s="40" t="inlineStr">
-        <is>
-          <t>SULEYMAN YILDIZ</t>
-        </is>
-      </c>
+      <c r="D36" s="6" t="n"/>
       <c r="E36" s="6" t="n"/>
       <c r="F36" s="6" t="n"/>
       <c r="G36" s="6" t="n"/>
@@ -1531,11 +1513,7 @@
           <t>09:00</t>
         </is>
       </c>
-      <c r="J36" s="41" t="inlineStr">
-        <is>
-          <t>SULEYMAN YILDIZ</t>
-        </is>
-      </c>
+      <c r="J36" s="9" t="n"/>
       <c r="K36" s="10" t="n"/>
     </row>
     <row r="37" ht="21.75" customHeight="1">
@@ -1547,11 +1525,7 @@
           <t>01:00</t>
         </is>
       </c>
-      <c r="D37" s="40" t="inlineStr">
-        <is>
-          <t>SULEYMAN YILDIZ</t>
-        </is>
-      </c>
+      <c r="D37" s="6" t="n"/>
       <c r="E37" s="6" t="n"/>
       <c r="F37" s="6" t="n"/>
       <c r="G37" s="6" t="n"/>
@@ -1561,11 +1535,7 @@
           <t>09:00</t>
         </is>
       </c>
-      <c r="J37" s="41" t="inlineStr">
-        <is>
-          <t>SULEYMAN YILDIZ</t>
-        </is>
-      </c>
+      <c r="J37" s="9" t="n"/>
       <c r="K37" s="10" t="n"/>
     </row>
     <row r="38" ht="21.75" customHeight="1">
@@ -1599,11 +1569,7 @@
           <t>17:00</t>
         </is>
       </c>
-      <c r="D39" s="40" t="inlineStr">
-        <is>
-          <t>SULEYMAN YILDIZ</t>
-        </is>
-      </c>
+      <c r="D39" s="6" t="n"/>
       <c r="E39" s="6" t="n"/>
       <c r="F39" s="6" t="n"/>
       <c r="G39" s="6" t="n"/>
@@ -1613,11 +1579,7 @@
           <t>01:00</t>
         </is>
       </c>
-      <c r="J39" s="41" t="inlineStr">
-        <is>
-          <t>SULEYMAN YILDIZ</t>
-        </is>
-      </c>
+      <c r="J39" s="9" t="n"/>
       <c r="K39" s="10" t="n"/>
     </row>
     <row r="40" ht="21.75" customHeight="1">
@@ -1629,11 +1591,7 @@
           <t>09:00</t>
         </is>
       </c>
-      <c r="D40" s="40" t="inlineStr">
-        <is>
-          <t>SULEYMAN YILDIZ</t>
-        </is>
-      </c>
+      <c r="D40" s="6" t="n"/>
       <c r="E40" s="6" t="n"/>
       <c r="F40" s="6" t="n"/>
       <c r="G40" s="6" t="n"/>
@@ -1643,11 +1601,7 @@
           <t>17:00</t>
         </is>
       </c>
-      <c r="J40" s="41" t="inlineStr">
-        <is>
-          <t>SULEYMAN YILDIZ</t>
-        </is>
-      </c>
+      <c r="J40" s="9" t="n"/>
       <c r="K40" s="10" t="n"/>
     </row>
     <row r="41" ht="21.75" customHeight="1">
@@ -1659,11 +1613,7 @@
           <t>09:00</t>
         </is>
       </c>
-      <c r="D41" s="40" t="inlineStr">
-        <is>
-          <t>SULEYMAN YILDIZ</t>
-        </is>
-      </c>
+      <c r="D41" s="6" t="n"/>
       <c r="E41" s="6" t="n"/>
       <c r="F41" s="6" t="n"/>
       <c r="G41" s="6" t="n"/>
@@ -1673,11 +1623,7 @@
           <t>17:00</t>
         </is>
       </c>
-      <c r="J41" s="41" t="inlineStr">
-        <is>
-          <t>SULEYMAN YILDIZ</t>
-        </is>
-      </c>
+      <c r="J41" s="9" t="n"/>
       <c r="K41" s="10" t="n"/>
     </row>
     <row r="42" ht="21.75" customHeight="1">
@@ -1689,11 +1635,7 @@
           <t>09:00</t>
         </is>
       </c>
-      <c r="D42" s="40" t="inlineStr">
-        <is>
-          <t>SULEYMAN YILDIZ</t>
-        </is>
-      </c>
+      <c r="D42" s="6" t="n"/>
       <c r="E42" s="6" t="n"/>
       <c r="F42" s="6" t="n"/>
       <c r="G42" s="6" t="n"/>
@@ -1703,11 +1645,7 @@
           <t>17:00</t>
         </is>
       </c>
-      <c r="J42" s="41" t="inlineStr">
-        <is>
-          <t>SULEYMAN YILDIZ</t>
-        </is>
-      </c>
+      <c r="J42" s="9" t="n"/>
       <c r="K42" s="10" t="n"/>
     </row>
     <row r="43" ht="21.75" customHeight="1">
@@ -1719,11 +1657,7 @@
           <t>09:00</t>
         </is>
       </c>
-      <c r="D43" s="40" t="inlineStr">
-        <is>
-          <t>SULEYMAN YILDIZ</t>
-        </is>
-      </c>
+      <c r="D43" s="6" t="n"/>
       <c r="E43" s="6" t="n"/>
       <c r="F43" s="6" t="n"/>
       <c r="G43" s="6" t="n"/>
@@ -1733,11 +1667,7 @@
           <t>17:00</t>
         </is>
       </c>
-      <c r="J43" s="41" t="inlineStr">
-        <is>
-          <t>SULEYMAN YILDIZ</t>
-        </is>
-      </c>
+      <c r="J43" s="9" t="n"/>
       <c r="K43" s="10" t="n"/>
     </row>
     <row r="44" ht="21.75" customHeight="1">
@@ -1749,11 +1679,7 @@
           <t>09:00</t>
         </is>
       </c>
-      <c r="D44" s="40" t="inlineStr">
-        <is>
-          <t>SULEYMAN YILDIZ</t>
-        </is>
-      </c>
+      <c r="D44" s="6" t="n"/>
       <c r="E44" s="6" t="n"/>
       <c r="F44" s="6" t="n"/>
       <c r="G44" s="6" t="n"/>
@@ -1763,11 +1689,7 @@
           <t>17:00</t>
         </is>
       </c>
-      <c r="J44" s="41" t="inlineStr">
-        <is>
-          <t>SULEYMAN YILDIZ</t>
-        </is>
-      </c>
+      <c r="J44" s="9" t="n"/>
       <c r="K44" s="10" t="n"/>
     </row>
     <row r="45" ht="21.75" customHeight="1" thickBot="1">

</xml_diff>

<commit_message>
Add September 2026 attendance sheets per person
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01LsGdck9uUBqMn7Bw6wMhA5
</commit_message>
<xml_diff>
--- a/Personel_Devam_Cizelgesi_Eylul_2026_SULEYMAN_YILDIZ.xlsx
+++ b/Personel_Devam_Cizelgesi_Eylul_2026_SULEYMAN_YILDIZ.xlsx
@@ -6,10 +6,10 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="0" showVerticalScroll="0" showSheetTabs="0" xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SULEYMAN YILDIZ" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SÜLEYMAN YILDIZ" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">'SULEYMAN YILDIZ'!$B$1:$K$46</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">'SÜLEYMAN YILDIZ'!$B$1:$K$46</definedName>
   </definedNames>
   <calcPr calcId="181029" fullCalcOnLoad="1"/>
 </workbook>
@@ -938,7 +938,7 @@
     <row r="4" ht="32.25" customHeight="1">
       <c r="B4" s="32" t="inlineStr">
         <is>
-          <t>Adı,Soyadı;  SULEYMAN YILDIZ</t>
+          <t>Adı,Soyadı;  SÜLEYMAN YILDIZ</t>
         </is>
       </c>
       <c r="C4" s="38" t="n"/>

</xml_diff>